<commit_message>
Clean dataset: fix titles, drop non-service pages, fill missing fields, split referents
</commit_message>
<xml_diff>
--- a/data/exports/services_overview.xlsx
+++ b/data/exports/services_overview.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Contacts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pages'!$A$1:$G$50</definedName>
@@ -956,19 +956,19 @@
 Heranführung von Kindern und Jugendlichen, Probleme demokratisch zu lösen, z.B. während eines Aufenthalts in einer Einrichtung
 Beratungsstellen der Caritas in Unterfranken:
 Erziehungsberatungsstelle Aschaffenburg
-Außensprechstunde Aschaffenburg - Schloßberg 4
-Außensprechstunde Alzenau - Beratungszentrum Alfred-Delp-Straße 4
+Außensprechstunde Aschaffenburg - Schloßberg 4
+Außensprechstunde Alzenau - Beratungszentrum Alfred-Delp-Straße 4
 Außensprechstunde Großostheim
 Treibgasse 26, 63739 Aschaffenburg
 06021 392-301
 Erziehungsberatungsstelle Bad Kissingen
-Außensprechstunde Bad Brückenau - Ernst-Putz-Straße 4a
-Außensprechstunde Hammelburg - von-Hess-Straße 18
+Außensprechstunde Bad Brückenau - Ernst-Putz-Straße 4a
+Außensprechstunde Hammelburg - von-Hess-Straße 18
 Außensprechstunde Wildflecken - Rathaus
 Hartmannstr. 2a, 97688 Bas Kissingen
 0971 7246-9200
 Erziehungsberatungsstelle Bad Neustadt / Saale
-Außensprechstunde Mellrichstadt
+Außensprechstunde Mellrichstadt
 Außensprechstunde Bad Königshofen
 Kellereigasse 12, 97616 Bad Neustadt
 09771 6116-15
@@ -977,8 +977,8 @@
 Obere Vorstadt 19, 97437 Haßfurt
 09521 69131
 Erziehungsberatungsstelle Kitzingen
-Außensprechstunde Stadtteilzentrum Kitzingen
-Außensprechstunde Volkach
+Außensprechstunde Stadtteilzentrum Kitzingen
+Außensprechstunde Volkach
 Güterhallstr. 5, 97318 Kitzingen
 09321 7817
 Erziehungsberatungsstelle Miltenberg
@@ -986,7 +986,7 @@
 Hauptstraße 60, 63897 Miltenberg
 09371 9789-20
 Erziehungsberatungsstelle Würzburg
-Außensprechstunde Giebelstadt - Obere Kirchgasse 6 - 09334 993242
+Außensprechstunde Giebelstadt - Obere Kirchgasse 6 - 09334 993242
 Außensprechstunde Ochsenfurt - Kellereistraße 8 - 0931 804570
 Frankfurter Str. 24, 97082 Würzburg
 0931 4190461
@@ -1757,7 +1757,7 @@
 Hilfreiche Adressen und Links
 Caritasverband für die Stadt und den Landkreis Würzburg e.V.
 Allgemeiner Sozialdienst
-Matthias-Ehrenfried-Haus,
+Matthias-Ehrenfried-Haus,
 Bahnhofstr. 4-6, 97070 Würzburg
 0931 386-59122 - Frau Hackel
 0931 386-59121 - Frau Berl
@@ -1765,8 +1765,8 @@
 http://www.caritas-wuerzburg.org/einrichtungen/allgemeiner-sozialdienst/
 Caritasverband für die Stadt und den Landkreis Aschaffenburg e.V.
 Allgemeiner Sozialer Beratungsdienst
-Martinushaus, 
-Treibgasse 26
+Martinushaus, 
+Treibgasse 26
 , 63739 Aschaffenburg
 06021 392-206
 06021 392-199
@@ -2476,7 +2476,7 @@
 http://www.diakonie-schweinfurt.de/rat-und-hilfe/sucht-und-abhaengigkeit
 Caritasverband für die Stadt und den Landkreis Würzburg e.V.
 Psychosoziale Beratungsstelle für Suchtprobleme/Fachstelle der Landesstelle Glücksspielsucht in Bayern - Suchtmittelkonsum und -abhängigkeit von legalen Suchtmitteln, Spielsucht, Essstörungen, Verhaltensabhängigkeiten
-Matthias-Ehrenfried-Haus
+Matthias-Ehrenfried-Haus
 Bahnhofstraße 4-6, 97070 Würzburg
 0931 38659180
 0931 38659189
@@ -2937,8 +2937,8 @@
 © BayStMI
 Ihr Ansprechpartner
 Rainer Jäckel
-Flüchtlings- und Integrationsberater
-Dienststellenleiter
+Flüchtlings- und Integrationsberater
+Dienststellenleiter
 Caritasverband für die Diözese Würzburg e.V.
 Dominikanerplatz 8, 97070 Würzburg
 0931 38658152
@@ -3338,7 +3338,7 @@
 Hier finden Sie für den Caritasverband Ansprechpartnerinnen und -partner im Bereich Prävention, Interventionskoordination und Aufarbeitung. Die Stabsstelle besteht aus folgenden Mitgliedern:
 Stefanie
  Eisenhuth
-Leitung der Stabsstelle
+Leitung der Stabsstelle
 Prävention, Interventionskoordination und Aufarbeitung
 Caritasverband für die Diözese Würzburg e. V.
 Franziskanergasse 3, 97070 Würzburg
@@ -3350,7 +3350,7 @@
 . 
 Florian
  Fell
-Prävention sexualisierter Gewalt
+Prävention sexualisierter Gewalt
 Kinder und Jugendliche
 Caritasverband für die Diözese Würzburg e. V.
 Franziskanergasse 3, 97070 Würzburg
@@ -3359,7 +3359,7 @@
 florian.fell@caritas-wuerzburg.de
 Tim
  Braunbeck
-Prävention sexualisierter Gewalt
+Prävention sexualisierter Gewalt
 Gesundheit und Alter
 Caritasverband für die Diözese Würzburg e. V.
 Franziskanergasse 3, 97070 Würzburg
@@ -3375,7 +3375,7 @@
 phyllis.kunad@caritas-wuerzburg.de
 Aaron
  Roth
-Studentische Hilfskraft der Stabstelle Prävention
+Studentische Hilfskraft der Stabstelle Prävention
 Caritasverband für die Diözese Würzburg e. V.
 Franziskanergasse 3, 97070 Würzburg
 0931 386-68941

</xml_diff>